<commit_message>
📊 Improve Table 2: consolidated format for journal papers
IMPROVEMENT: Better detection table format for publications

Changes:
- ❌ OLD: 4 separate sheets (hard to compare)
- ✅ NEW: Single consolidated table with Dataset column

New Format:
- All 12 results (4 datasets × 3 models) in ONE view
- Dataset column for easy comparison across datasets
- Better for journal papers: direct cross-dataset comparison
- Easier to copy-paste to Word/LaTeX

New Script:
- scripts/reporting/generate_table2_detection_consolidated.py
- Generates single-sheet consolidated detection table
- Grouped styling per dataset (alternating colors)

Benefits:
✓ All data visible at once (no sheet switching)
✓ Easy comparison: YOLO10 vs YOLO11 vs YOLO12
✓ Easy comparison across datasets
✓ Standard academic journal format
✓ Better for publication submission

User Request: 'tabel 2 kenapa tidak ada breakdown untuk per dataset nya'
Answer: Now has Dataset column for clear breakdown!
</commit_message>
<xml_diff>
--- a/luaran/laporan_akhir/tables/Table2_Detection_Performance.xlsx
+++ b/luaran/laporan_akhir/tables/Table2_Detection_Performance.xlsx
@@ -7,10 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="IML Lifecycle" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="MP-IDB Species" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="MP-IDB Stages" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="MD-2019 Stages" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Detection Performance" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
     <font>
       <b val="1"/>
@@ -57,19 +51,13 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
-    </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
     </border>
     <border>
       <left style="thin">
@@ -89,21 +77,27 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="2" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="1" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -471,44 +465,50 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>Dataset</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>mAP@50 (%)</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>mAP@50-95 (%)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Precision (%)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Recall (%)</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Best Epoch</t>
         </is>
@@ -517,426 +517,324 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
+          <t>IML Lifecycle</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
           <t>YOLO10</t>
         </is>
       </c>
-      <c r="B2" s="3" t="n">
-        <v>0.9602000000000001</v>
-      </c>
       <c r="C2" s="3" t="n">
-        <v>0.7734</v>
+        <v>96.02000000000001</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0.8912</v>
+        <v>77.34</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>0.9287</v>
+        <v>89.12</v>
       </c>
       <c r="F2" s="3" t="n">
+        <v>92.86999999999999</v>
+      </c>
+      <c r="G2" s="4" t="n">
         <v>23</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>IML Lifecycle</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>YOLO11</t>
         </is>
       </c>
-      <c r="B3" s="5" t="n">
-        <v>0.9661</v>
-      </c>
-      <c r="C3" s="5" t="n">
-        <v>0.7319</v>
-      </c>
-      <c r="D3" s="5" t="n">
-        <v>0.8617</v>
-      </c>
-      <c r="E3" s="5" t="n">
-        <v>0.9588</v>
-      </c>
-      <c r="F3" s="5" t="n">
+      <c r="C3" s="3" t="n">
+        <v>96.61</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>73.19</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>86.17</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>95.88</v>
+      </c>
+      <c r="G3" s="4" t="n">
         <v>18</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
+          <t>IML Lifecycle</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
           <t>YOLO12</t>
         </is>
       </c>
-      <c r="B4" s="3" t="n">
-        <v>0.9616</v>
-      </c>
       <c r="C4" s="3" t="n">
-        <v>0.7801</v>
+        <v>96.16</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>0.8938</v>
+        <v>78.01000000000001</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>0.9278</v>
+        <v>89.38000000000001</v>
       </c>
       <c r="F4" s="3" t="n">
+        <v>92.78</v>
+      </c>
+      <c r="G4" s="4" t="n">
         <v>47</v>
       </c>
     </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Model</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>mAP@50 (%)</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>mAP@50-95 (%)</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Precision (%)</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Recall (%)</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Best Epoch</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>MP-IDB Species</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>YOLO10</t>
         </is>
       </c>
-      <c r="B2" s="3" t="n">
-        <v>0.9468</v>
-      </c>
-      <c r="C2" s="3" t="n">
-        <v>0.6151</v>
-      </c>
-      <c r="D2" s="3" t="n">
-        <v>0.9174</v>
-      </c>
-      <c r="E2" s="3" t="n">
-        <v>0.9125</v>
-      </c>
-      <c r="F2" s="3" t="n">
+      <c r="C5" s="6" t="n">
+        <v>94.67999999999999</v>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>61.51</v>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>91.73999999999999</v>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>91.25</v>
+      </c>
+      <c r="G5" s="7" t="n">
         <v>67</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>MP-IDB Species</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>YOLO11</t>
         </is>
       </c>
-      <c r="B3" s="5" t="n">
-        <v>0.9656</v>
-      </c>
-      <c r="C3" s="5" t="n">
-        <v>0.6374</v>
-      </c>
-      <c r="D3" s="5" t="n">
-        <v>0.9009</v>
-      </c>
-      <c r="E3" s="5" t="n">
-        <v>0.9529</v>
-      </c>
-      <c r="F3" s="5" t="n">
+      <c r="C6" s="6" t="n">
+        <v>96.56</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>63.73999999999999</v>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>90.09</v>
+      </c>
+      <c r="F6" s="6" t="n">
+        <v>95.28999999999999</v>
+      </c>
+      <c r="G6" s="7" t="n">
         <v>86</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>MP-IDB Species</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>YOLO12</t>
         </is>
       </c>
-      <c r="B4" s="3" t="n">
-        <v>0.9569</v>
-      </c>
-      <c r="C4" s="3" t="n">
-        <v>0.6274</v>
-      </c>
-      <c r="D4" s="3" t="n">
-        <v>0.9438</v>
-      </c>
-      <c r="E4" s="3" t="n">
-        <v>0.8956</v>
-      </c>
-      <c r="F4" s="3" t="n">
+      <c r="C7" s="6" t="n">
+        <v>95.69</v>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>62.73999999999999</v>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>94.38</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>89.56</v>
+      </c>
+      <c r="G7" s="7" t="n">
         <v>84</v>
       </c>
     </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Model</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>mAP@50 (%)</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>mAP@50-95 (%)</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Precision (%)</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Recall (%)</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Best Epoch</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>MP-IDB Stages</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>YOLO10</t>
         </is>
       </c>
-      <c r="B2" s="3" t="n">
-        <v>0.9186</v>
-      </c>
-      <c r="C2" s="3" t="n">
-        <v>0.5272</v>
-      </c>
-      <c r="D2" s="3" t="n">
-        <v>0.9022</v>
-      </c>
-      <c r="E2" s="3" t="n">
-        <v>0.8964</v>
-      </c>
-      <c r="F2" s="3" t="n">
+      <c r="C8" s="3" t="n">
+        <v>91.86</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>52.72</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>90.22</v>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>89.64</v>
+      </c>
+      <c r="G8" s="4" t="n">
         <v>96</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>MP-IDB Stages</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>YOLO11</t>
         </is>
       </c>
-      <c r="B3" s="5" t="n">
-        <v>0.9335</v>
-      </c>
-      <c r="C3" s="5" t="n">
-        <v>0.4778</v>
-      </c>
-      <c r="D3" s="5" t="n">
-        <v>0.8925999999999999</v>
-      </c>
-      <c r="E3" s="5" t="n">
-        <v>0.9086</v>
-      </c>
-      <c r="F3" s="5" t="n">
+      <c r="C9" s="3" t="n">
+        <v>93.34999999999999</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>47.78</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>89.25999999999999</v>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>90.86</v>
+      </c>
+      <c r="G9" s="4" t="n">
         <v>67</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>MP-IDB Stages</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>YOLO12</t>
         </is>
       </c>
-      <c r="B4" s="3" t="n">
-        <v>0.9562</v>
-      </c>
-      <c r="C4" s="3" t="n">
-        <v>0.5891</v>
-      </c>
-      <c r="D4" s="3" t="n">
-        <v>0.9216</v>
-      </c>
-      <c r="E4" s="3" t="n">
-        <v>0.9143</v>
-      </c>
-      <c r="F4" s="3" t="n">
+      <c r="C10" s="3" t="n">
+        <v>95.62</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>58.91</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>92.16</v>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>91.43000000000001</v>
+      </c>
+      <c r="G10" s="4" t="n">
         <v>95</v>
       </c>
     </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Model</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>mAP@50 (%)</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>mAP@50-95 (%)</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Precision (%)</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Recall (%)</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Best Epoch</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>MD-2019 Stages</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>YOLO10</t>
         </is>
       </c>
-      <c r="B2" s="3" t="n">
-        <v>0.9274</v>
-      </c>
-      <c r="C2" s="3" t="n">
-        <v>0.7055</v>
-      </c>
-      <c r="D2" s="3" t="n">
-        <v>0.8178</v>
-      </c>
-      <c r="E2" s="3" t="n">
-        <v>0.8947000000000001</v>
-      </c>
-      <c r="F2" s="3" t="n">
+      <c r="C11" s="6" t="n">
+        <v>92.73999999999999</v>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>70.55</v>
+      </c>
+      <c r="E11" s="6" t="n">
+        <v>81.78</v>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>89.47</v>
+      </c>
+      <c r="G11" s="7" t="n">
         <v>26</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>MD-2019 Stages</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>YOLO11</t>
         </is>
       </c>
-      <c r="B3" s="5" t="n">
-        <v>0.9298</v>
-      </c>
-      <c r="C3" s="5" t="n">
-        <v>0.7726</v>
-      </c>
-      <c r="D3" s="5" t="n">
-        <v>0.8433</v>
-      </c>
-      <c r="E3" s="5" t="n">
-        <v>0.8709</v>
-      </c>
-      <c r="F3" s="5" t="n">
+      <c r="C12" s="6" t="n">
+        <v>92.97999999999999</v>
+      </c>
+      <c r="D12" s="6" t="n">
+        <v>77.25999999999999</v>
+      </c>
+      <c r="E12" s="6" t="n">
+        <v>84.33</v>
+      </c>
+      <c r="F12" s="6" t="n">
+        <v>87.09</v>
+      </c>
+      <c r="G12" s="7" t="n">
         <v>54</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>MD-2019 Stages</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>YOLO12</t>
         </is>
       </c>
-      <c r="B4" s="3" t="n">
-        <v>0.9346</v>
-      </c>
-      <c r="C4" s="3" t="n">
-        <v>0.7754</v>
-      </c>
-      <c r="D4" s="3" t="n">
-        <v>0.8782</v>
-      </c>
-      <c r="E4" s="3" t="n">
-        <v>0.8421</v>
-      </c>
-      <c r="F4" s="3" t="n">
+      <c r="C13" s="6" t="n">
+        <v>93.45999999999999</v>
+      </c>
+      <c r="D13" s="6" t="n">
+        <v>77.53999999999999</v>
+      </c>
+      <c r="E13" s="6" t="n">
+        <v>87.81999999999999</v>
+      </c>
+      <c r="F13" s="6" t="n">
+        <v>84.20999999999999</v>
+      </c>
+      <c r="G13" s="7" t="n">
         <v>64</v>
       </c>
     </row>

</xml_diff>